<commit_message>
Added outer square but it doesn't work yet
</commit_message>
<xml_diff>
--- a/20260414-King is Dead Adjacency.xlsx
+++ b/20260414-King is Dead Adjacency.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\nick\Desktop\board_game_maps\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{208385FB-5890-4278-9295-2AC490668978}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDC9192F-0EA2-420E-9267-1C0B07270331}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4290" yWindow="2865" windowWidth="28800" windowHeight="15435" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1665" yWindow="2970" windowWidth="28800" windowHeight="15435" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="8">
   <si>
     <t>Moray</t>
   </si>
@@ -49,9 +49,6 @@
   </si>
   <si>
     <t>Northumbria</t>
-  </si>
-  <si>
-    <t>Sea</t>
   </si>
 </sst>
 </file>
@@ -369,10 +366,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -397,11 +394,8 @@
       <c r="I1" t="s">
         <v>6</v>
       </c>
-      <c r="J1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -429,11 +423,8 @@
       <c r="I2">
         <v>0</v>
       </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -461,11 +452,8 @@
       <c r="I3">
         <v>0</v>
       </c>
-      <c r="J3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -493,11 +481,8 @@
       <c r="I4">
         <v>0</v>
       </c>
-      <c r="J4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -525,11 +510,8 @@
       <c r="I5">
         <v>0</v>
       </c>
-      <c r="J5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -557,11 +539,8 @@
       <c r="I6">
         <v>1</v>
       </c>
-      <c r="J6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -589,11 +568,8 @@
       <c r="I7">
         <v>1</v>
       </c>
-      <c r="J7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -621,11 +597,8 @@
       <c r="I8">
         <v>1</v>
       </c>
-      <c r="J8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -651,41 +624,6 @@
         <v>1</v>
       </c>
       <c r="I9">
-        <v>0</v>
-      </c>
-      <c r="J9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10">
-        <v>1</v>
-      </c>
-      <c r="C10">
-        <v>1</v>
-      </c>
-      <c r="D10">
-        <v>1</v>
-      </c>
-      <c r="E10">
-        <v>1</v>
-      </c>
-      <c r="F10">
-        <v>1</v>
-      </c>
-      <c r="G10">
-        <v>0</v>
-      </c>
-      <c r="H10">
-        <v>1</v>
-      </c>
-      <c r="I10">
-        <v>1</v>
-      </c>
-      <c r="J10">
         <v>0</v>
       </c>
     </row>

</xml_diff>